<commit_message>
Fix: swap spiritMedicineOfficialOutline[2]/[3] xlsx data to match reordered TS array
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/page-copy/05-视频目录-灵体医学.xlsx
+++ b/docs/page-copy/05-视频目录-灵体医学.xlsx
@@ -2041,7 +2041,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>spiritMedicineOfficialOutline[2].fileLabel</v>
+        <v>spiritMedicineOfficialOutline[3].fileLabel</v>
       </c>
       <c r="B72" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2064,7 +2064,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>spiritMedicineOfficialOutline[2].heading</v>
+        <v>spiritMedicineOfficialOutline[3].heading</v>
       </c>
       <c r="B73" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2087,7 +2087,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>spiritMedicineOfficialOutline[2].subsections[0].code</v>
+        <v>spiritMedicineOfficialOutline[3].subsections[0].code</v>
       </c>
       <c r="B74" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2110,7 +2110,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>spiritMedicineOfficialOutline[2].subsections[0].title</v>
+        <v>spiritMedicineOfficialOutline[3].subsections[0].title</v>
       </c>
       <c r="B75" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2133,7 +2133,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>spiritMedicineOfficialOutline[2].subsections[1].code</v>
+        <v>spiritMedicineOfficialOutline[3].subsections[1].code</v>
       </c>
       <c r="B76" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2156,7 +2156,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>spiritMedicineOfficialOutline[2].subsections[1].title</v>
+        <v>spiritMedicineOfficialOutline[3].subsections[1].title</v>
       </c>
       <c r="B77" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2179,7 +2179,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>spiritMedicineOfficialOutline[3].fileLabel</v>
+        <v>spiritMedicineOfficialOutline[2].fileLabel</v>
       </c>
       <c r="B78" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2202,7 +2202,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>spiritMedicineOfficialOutline[3].heading</v>
+        <v>spiritMedicineOfficialOutline[2].heading</v>
       </c>
       <c r="B79" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2225,7 +2225,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>spiritMedicineOfficialOutline[3].subsections[0].code</v>
+        <v>spiritMedicineOfficialOutline[2].subsections[0].code</v>
       </c>
       <c r="B80" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2248,7 +2248,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>spiritMedicineOfficialOutline[3].subsections[0].title</v>
+        <v>spiritMedicineOfficialOutline[2].subsections[0].title</v>
       </c>
       <c r="B81" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2271,7 +2271,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>spiritMedicineOfficialOutline[3].subsections[1].code</v>
+        <v>spiritMedicineOfficialOutline[2].subsections[1].code</v>
       </c>
       <c r="B82" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2294,7 +2294,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>spiritMedicineOfficialOutline[3].subsections[1].title</v>
+        <v>spiritMedicineOfficialOutline[2].subsections[1].title</v>
       </c>
       <c r="B83" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2317,7 +2317,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>spiritMedicineOfficialOutline[3].subsections[2].code</v>
+        <v>spiritMedicineOfficialOutline[2].subsections[2].code</v>
       </c>
       <c r="B84" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2340,7 +2340,7 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>spiritMedicineOfficialOutline[3].subsections[2].title</v>
+        <v>spiritMedicineOfficialOutline[2].subsections[2].title</v>
       </c>
       <c r="B85" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2363,7 +2363,7 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>spiritMedicineOfficialOutline[3].subsections[3].code</v>
+        <v>spiritMedicineOfficialOutline[2].subsections[3].code</v>
       </c>
       <c r="B86" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2386,7 +2386,7 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>spiritMedicineOfficialOutline[3].subsections[3].title</v>
+        <v>spiritMedicineOfficialOutline[2].subsections[3].title</v>
       </c>
       <c r="B87" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2409,7 +2409,7 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>spiritMedicineOfficialOutline[3].subsections[4].code</v>
+        <v>spiritMedicineOfficialOutline[2].subsections[4].code</v>
       </c>
       <c r="B88" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2432,7 +2432,7 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>spiritMedicineOfficialOutline[3].subsections[4].title</v>
+        <v>spiritMedicineOfficialOutline[2].subsections[4].title</v>
       </c>
       <c r="B89" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2455,7 +2455,7 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>spiritMedicineOfficialOutline[3].subsections[5].code</v>
+        <v>spiritMedicineOfficialOutline[2].subsections[5].code</v>
       </c>
       <c r="B90" t="str">
         <v>灵体医学 / 完整目录</v>
@@ -2478,7 +2478,7 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>spiritMedicineOfficialOutline[3].subsections[5].title</v>
+        <v>spiritMedicineOfficialOutline[2].subsections[5].title</v>
       </c>
       <c r="B91" t="str">
         <v>灵体医学 / 完整目录</v>

</xml_diff>